<commit_message>
Improve MICE safety decision briefs
</commit_message>
<xml_diff>
--- a/outputs/may-2026-real-events/details/02-kintex-playx4-2026/bundle/tables/safety-checklists.xlsx
+++ b/outputs/may-2026-real-events/details/02-kintex-playx4-2026/bundle/tables/safety-checklists.xlsx
@@ -7947,7 +7947,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>작업책임자</t>
+          <t>공연안전 담당</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7957,17 +7957,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>시공/하역/전기 협력사</t>
+          <t>공연/문화 담당부서·베뉴 기술지원</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>운영본부/구역장</t>
+          <t>운영본부/무대감독/보안·의료팀</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>작업계획서/교육명단/PPE 지급/작업허가·작업중지 기준</t>
+          <t>공연 재해대처계획/안전교육 명단/무대·리깅 승인/공연중지 기준</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -8101,7 +8101,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>소방·피난 점검표/위험물 반입 승인/개장 전 사진</t>
+          <t>베뉴 제출 승인서/부스·전기 신청서/반입·하역 승인/현장 확인 사진</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">

</xml_diff>